<commit_message>
Split out bigint.c into a 32 and 64-bit version, used in the appropriate build, after it was decided that it's too hard to get a unified source, especially for the mult and div routines.
</commit_message>
<xml_diff>
--- a/Benchmarks.xlsx
+++ b/Benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\bigint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{539396C0-BD5F-4E42-BC7A-360A6E3770C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47695910-0EC7-4267-AB19-4AD7AB73DAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="14730" xr2:uid="{04B2B848-95FC-4839-9E9B-95D007D1E4DA}"/>
+    <workbookView xWindow="6210" yWindow="405" windowWidth="21600" windowHeight="14730" xr2:uid="{04B2B848-95FC-4839-9E9B-95D007D1E4DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -62,10 +62,10 @@
     <t>x86 (32-bit)</t>
   </si>
   <si>
-    <t>1M additions:</t>
-  </si>
-  <si>
     <t>Using intrinsics (_addcarry_u32, _subborrow_u32, etc)</t>
+  </si>
+  <si>
+    <t>Subtraction:</t>
   </si>
 </sst>
 </file>
@@ -446,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22329E99-4E70-452E-B5ED-3C6372A6D317}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
@@ -472,19 +472,19 @@
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="1">
         <v>10</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="1">
         <v>30</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>100</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="1">
         <v>500</v>
       </c>
       <c r="F4">
@@ -495,146 +495,153 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5">
-        <v>28</v>
-      </c>
-      <c r="C5">
-        <v>28</v>
-      </c>
-      <c r="D5">
-        <v>29</v>
-      </c>
-      <c r="E5">
-        <v>41</v>
-      </c>
-      <c r="F5">
-        <v>72</v>
-      </c>
-      <c r="G5">
-        <v>109</v>
-      </c>
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="C6">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="D6">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="E6">
-        <v>256</v>
+        <v>125</v>
       </c>
       <c r="F6">
-        <v>3100</v>
+        <v>298</v>
       </c>
       <c r="G6">
-        <v>18083</v>
+        <v>535</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B7">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C7">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="D7">
-        <v>111</v>
+        <v>71</v>
       </c>
       <c r="E7">
-        <v>415</v>
+        <v>136</v>
       </c>
       <c r="F7">
-        <v>3016</v>
+        <v>308</v>
       </c>
       <c r="G7">
-        <v>12271</v>
+        <v>526</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8">
         <v>7</v>
       </c>
-      <c r="B8">
-        <v>271</v>
-      </c>
-      <c r="C8">
-        <v>276</v>
-      </c>
       <c r="D8">
-        <v>304</v>
+        <v>12</v>
       </c>
       <c r="E8">
-        <v>406</v>
+        <v>97</v>
       </c>
       <c r="F8">
-        <v>679</v>
+        <v>1237</v>
       </c>
       <c r="G8">
-        <v>1084</v>
+        <v>7297</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>21</v>
+      </c>
+      <c r="D9">
+        <v>33</v>
+      </c>
+      <c r="E9">
+        <v>177</v>
+      </c>
+      <c r="F9">
+        <v>1290</v>
+      </c>
+      <c r="G9">
+        <v>5024</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12">
+        <v>54</v>
+      </c>
+      <c r="C12">
+        <v>53</v>
+      </c>
+      <c r="D12">
+        <v>61</v>
+      </c>
+      <c r="E12">
+        <v>94</v>
+      </c>
+      <c r="F12">
+        <v>208</v>
+      </c>
+      <c r="G12">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10">
-        <v>27</v>
-      </c>
-      <c r="C10">
-        <v>28</v>
-      </c>
-      <c r="D10">
-        <v>30</v>
-      </c>
-      <c r="E10">
-        <v>41</v>
-      </c>
-      <c r="F10">
-        <v>64</v>
-      </c>
-      <c r="G10">
+      <c r="B13">
+        <v>55</v>
+      </c>
+      <c r="C13">
+        <v>55</v>
+      </c>
+      <c r="D13">
+        <v>63</v>
+      </c>
+      <c r="E13">
         <v>95</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11">
-        <v>274</v>
-      </c>
-      <c r="C11">
-        <v>293</v>
-      </c>
-      <c r="D11">
-        <v>304</v>
-      </c>
-      <c r="E11">
-        <v>420</v>
-      </c>
-      <c r="F11">
-        <v>642</v>
-      </c>
-      <c r="G11">
-        <v>955</v>
+      <c r="F13">
+        <v>195</v>
+      </c>
+      <c r="G13">
+        <v>367</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Testing of x64 build with all but division converted over to intrinsics. Benchmarking shows it's a belter! Division may not be as impressive, though.
</commit_message>
<xml_diff>
--- a/Benchmarks.xlsx
+++ b/Benchmarks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\bigint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47695910-0EC7-4267-AB19-4AD7AB73DAF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C922A865-118B-4596-BF74-A43A6C95B9CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6210" yWindow="405" windowWidth="21600" windowHeight="14730" xr2:uid="{04B2B848-95FC-4839-9E9B-95D007D1E4DA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
   <si>
     <t>Original code</t>
   </si>
@@ -66,6 +66,12 @@
   </si>
   <si>
     <t>Subtraction:</t>
+  </si>
+  <si>
+    <t>(no division yet for x64 - it's just too hard to convert)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x64 build, with intrinsics </t>
   </si>
 </sst>
 </file>
@@ -446,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22329E99-4E70-452E-B5ED-3C6372A6D317}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
@@ -644,6 +650,85 @@
         <v>367</v>
       </c>
     </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>2</v>
+      </c>
+      <c r="B17">
+        <v>38</v>
+      </c>
+      <c r="C17">
+        <v>40</v>
+      </c>
+      <c r="D17">
+        <v>41</v>
+      </c>
+      <c r="E17">
+        <v>50</v>
+      </c>
+      <c r="F17">
+        <v>89</v>
+      </c>
+      <c r="G17">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18">
+        <v>38</v>
+      </c>
+      <c r="C18">
+        <v>43</v>
+      </c>
+      <c r="D18">
+        <v>40</v>
+      </c>
+      <c r="E18">
+        <v>54</v>
+      </c>
+      <c r="F18">
+        <v>87</v>
+      </c>
+      <c r="G18">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>3</v>
+      </c>
+      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="C19">
+        <v>4</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19">
+        <v>21</v>
+      </c>
+      <c r="F19">
+        <v>224</v>
+      </c>
+      <c r="G19">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Get rid of repeated malloc/free by ensuring that any routine giving a result bigint reuses its integer array wherever possible. This removes malloc/free time from contaminating the benchmark results, esp for small array sizes.
</commit_message>
<xml_diff>
--- a/Benchmarks.xlsx
+++ b/Benchmarks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\bigint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C922A865-118B-4596-BF74-A43A6C95B9CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70574C18-7066-442E-936B-ECB4F5958AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6210" yWindow="405" windowWidth="21600" windowHeight="14730" xr2:uid="{04B2B848-95FC-4839-9E9B-95D007D1E4DA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="11">
   <si>
     <t>Original code</t>
   </si>
@@ -452,7 +452,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22329E99-4E70-452E-B5ED-3C6372A6D317}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="1"/>
@@ -609,22 +609,22 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>54</v>
+        <v>5</v>
       </c>
       <c r="C12">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="D12">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="E12">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="F12">
-        <v>208</v>
+        <v>138</v>
       </c>
       <c r="G12">
-        <v>396</v>
+        <v>300</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -632,100 +632,146 @@
         <v>8</v>
       </c>
       <c r="B13">
-        <v>55</v>
+        <v>7</v>
       </c>
       <c r="C13">
-        <v>55</v>
+        <v>7</v>
       </c>
       <c r="D13">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="E13">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="F13">
-        <v>195</v>
+        <v>111</v>
       </c>
       <c r="G13">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14">
+        <v>6</v>
+      </c>
+      <c r="C14">
+        <v>7</v>
+      </c>
+      <c r="D14">
+        <v>12</v>
+      </c>
+      <c r="E14">
+        <v>106</v>
+      </c>
+      <c r="F14">
+        <v>1244</v>
+      </c>
+      <c r="G14">
+        <v>7294</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15">
+        <v>16</v>
+      </c>
+      <c r="D15">
+        <v>28</v>
+      </c>
+      <c r="E15">
+        <v>174</v>
+      </c>
+      <c r="F15">
+        <v>1294</v>
+      </c>
+      <c r="G15">
+        <v>5034</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>2</v>
-      </c>
-      <c r="B17">
-        <v>38</v>
-      </c>
-      <c r="C17">
-        <v>40</v>
-      </c>
-      <c r="D17">
-        <v>41</v>
-      </c>
-      <c r="E17">
-        <v>50</v>
-      </c>
-      <c r="F17">
-        <v>89</v>
-      </c>
-      <c r="G17">
-        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B18">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="C18">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="D18">
-        <v>40</v>
+        <v>7</v>
       </c>
       <c r="E18">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="F18">
-        <v>87</v>
+        <v>52</v>
       </c>
       <c r="G18">
-        <v>134</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19">
         <v>4</v>
       </c>
       <c r="D19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E19">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F19">
-        <v>224</v>
+        <v>51</v>
       </c>
       <c r="G19">
-        <v>1175</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20">
+        <v>4</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
+        <v>5</v>
+      </c>
+      <c r="E20">
+        <v>18</v>
+      </c>
+      <c r="F20">
+        <v>213</v>
+      </c>
+      <c r="G20">
+        <v>1189</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Backup. Move div64 back into main directory and integrate into bigint. Investigate slowdown (esp on 32-bit multiplies)
</commit_message>
<xml_diff>
--- a/Benchmarks.xlsx
+++ b/Benchmarks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\bigint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70574C18-7066-442E-936B-ECB4F5958AF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A16C4DA-9A8D-45C6-9549-F6A278FE6581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6210" yWindow="405" windowWidth="21600" windowHeight="14730" xr2:uid="{04B2B848-95FC-4839-9E9B-95D007D1E4DA}"/>
+    <workbookView xWindow="29910" yWindow="300" windowWidth="21600" windowHeight="14730" xr2:uid="{04B2B848-95FC-4839-9E9B-95D007D1E4DA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
   <si>
     <t>Original code</t>
   </si>
@@ -66,9 +66,6 @@
   </si>
   <si>
     <t>Subtraction:</t>
-  </si>
-  <si>
-    <t>(no division yet for x64 - it's just too hard to convert)</t>
   </si>
   <si>
     <t xml:space="preserve">x64 build, with intrinsics </t>
@@ -604,101 +601,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12">
-        <v>5</v>
-      </c>
-      <c r="C12">
-        <v>6</v>
-      </c>
-      <c r="D12">
-        <v>11</v>
-      </c>
-      <c r="E12">
-        <v>42</v>
-      </c>
-      <c r="F12">
-        <v>138</v>
-      </c>
-      <c r="G12">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>8</v>
-      </c>
-      <c r="B13">
-        <v>7</v>
-      </c>
-      <c r="C13">
-        <v>7</v>
-      </c>
-      <c r="D13">
-        <v>12</v>
-      </c>
-      <c r="E13">
-        <v>39</v>
-      </c>
-      <c r="F13">
-        <v>111</v>
-      </c>
-      <c r="G13">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14">
-        <v>6</v>
-      </c>
-      <c r="C14">
-        <v>7</v>
-      </c>
-      <c r="D14">
-        <v>12</v>
-      </c>
-      <c r="E14">
-        <v>106</v>
-      </c>
-      <c r="F14">
-        <v>1244</v>
-      </c>
-      <c r="G14">
-        <v>7294</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15">
-        <v>2</v>
-      </c>
-      <c r="C15">
-        <v>16</v>
-      </c>
-      <c r="D15">
-        <v>28</v>
-      </c>
-      <c r="E15">
-        <v>174</v>
-      </c>
-      <c r="F15">
-        <v>1294</v>
-      </c>
-      <c r="G15">
-        <v>5034</v>
-      </c>
-    </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -706,22 +611,22 @@
         <v>2</v>
       </c>
       <c r="B18">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C18">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D18">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E18">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="F18">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="G18">
-        <v>101</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -729,22 +634,22 @@
         <v>8</v>
       </c>
       <c r="B19">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C19">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D19">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E19">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="F19">
-        <v>51</v>
+        <v>98</v>
       </c>
       <c r="G19">
-        <v>101</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -752,27 +657,45 @@
         <v>3</v>
       </c>
       <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20">
+        <v>2</v>
+      </c>
+      <c r="D20">
         <v>4</v>
       </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20">
-        <v>5</v>
-      </c>
       <c r="E20">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F20">
-        <v>213</v>
+        <v>332</v>
       </c>
       <c r="G20">
-        <v>1189</v>
+        <v>1642</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>5</v>
+      </c>
+      <c r="B21">
+        <v>2</v>
+      </c>
+      <c r="C21">
+        <v>4</v>
+      </c>
+      <c r="D21">
+        <v>29</v>
+      </c>
+      <c r="E21">
+        <v>191</v>
+      </c>
+      <c r="F21">
+        <v>1469</v>
+      </c>
+      <c r="G21">
+        <v>5893</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tidy up. Express 32x32 multiply in intrinsics (which made no difference, unlike the 64-bit case). Add a 128x64 multiply operator to the uint128_t class to save time on some ops (again little difference)
</commit_message>
<xml_diff>
--- a/Benchmarks.xlsx
+++ b/Benchmarks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\bigint\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A16C4DA-9A8D-45C6-9549-F6A278FE6581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2E909CE-1172-408E-8401-0FF50B4BB8FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29910" yWindow="300" windowWidth="21600" windowHeight="14730" xr2:uid="{04B2B848-95FC-4839-9E9B-95D007D1E4DA}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
   <si>
     <t>Original code</t>
   </si>
@@ -601,6 +601,98 @@
         <v>7</v>
       </c>
     </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12">
+        <v>6</v>
+      </c>
+      <c r="C12">
+        <v>8</v>
+      </c>
+      <c r="D12">
+        <v>15</v>
+      </c>
+      <c r="E12">
+        <v>49</v>
+      </c>
+      <c r="F12">
+        <v>180</v>
+      </c>
+      <c r="G12">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13">
+        <v>8</v>
+      </c>
+      <c r="C13">
+        <v>9</v>
+      </c>
+      <c r="D13">
+        <v>14</v>
+      </c>
+      <c r="E13">
+        <v>48</v>
+      </c>
+      <c r="F13">
+        <v>122</v>
+      </c>
+      <c r="G13">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14">
+        <v>2</v>
+      </c>
+      <c r="D14">
+        <v>8</v>
+      </c>
+      <c r="E14">
+        <v>97</v>
+      </c>
+      <c r="F14">
+        <v>1281</v>
+      </c>
+      <c r="G14">
+        <v>7732</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15">
+        <v>17</v>
+      </c>
+      <c r="D15">
+        <v>31</v>
+      </c>
+      <c r="E15">
+        <v>175</v>
+      </c>
+      <c r="F15">
+        <v>1313</v>
+      </c>
+      <c r="G15">
+        <v>5211</v>
+      </c>
+    </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>9</v>
@@ -611,22 +703,22 @@
         <v>2</v>
       </c>
       <c r="B18">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C18">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D18">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E18">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F18">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="G18">
-        <v>161</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -634,22 +726,22 @@
         <v>8</v>
       </c>
       <c r="B19">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C19">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D19">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E19">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F19">
-        <v>98</v>
+        <v>55</v>
       </c>
       <c r="G19">
-        <v>191</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -657,22 +749,22 @@
         <v>3</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20">
         <v>2</v>
       </c>
-      <c r="D20">
-        <v>4</v>
-      </c>
       <c r="E20">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="F20">
-        <v>332</v>
+        <v>199</v>
       </c>
       <c r="G20">
-        <v>1642</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -680,22 +772,22 @@
         <v>5</v>
       </c>
       <c r="B21">
+        <v>1</v>
+      </c>
+      <c r="C21">
         <v>2</v>
       </c>
-      <c r="C21">
-        <v>4</v>
-      </c>
       <c r="D21">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E21">
-        <v>191</v>
+        <v>129</v>
       </c>
       <c r="F21">
-        <v>1469</v>
+        <v>1014</v>
       </c>
       <c r="G21">
-        <v>5893</v>
+        <v>4053</v>
       </c>
     </row>
   </sheetData>

</xml_diff>